<commit_message>
scan: seg6 2026-08-17 18:52 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-08-17.xlsx
+++ b/output/full_scan/batch_seq7_2026-08-17.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6092,38 +6092,38 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6654</v>
+        <v>6531</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>天正國際</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>221.1410406311564</v>
+        <v>221.2707713435213</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>176</v>
+        <v>873</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G107" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>51.7767829071333</v>
+        <v>50.97568761876995</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.43588992683855</v>
+        <v>13.38066165014582</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.8642299029807666</v>
+        <v>0.451535461460031</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,48 +6135,48 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>1.629373791420858</v>
+        <v>17.55233575479878</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6695</v>
+        <v>6654</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>天正國際</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>206.4841522859249</v>
+        <v>221.1410406311564</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>50.2</v>
+        <v>176</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G108" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>45.67018359258921</v>
+        <v>51.7767829071333</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>14.14828693055786</v>
+        <v>17.43588992683855</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.2998348168701576</v>
+        <v>0.8642299029807666</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.2779997355795514</v>
+        <v>1.629373791420858</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6790</v>
+        <v>6695</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>永豐實</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>201.3433314012784</v>
+        <v>206.4841522859249</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>37.9</v>
+        <v>50.2</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>35.57018055996438</v>
+        <v>45.67018359258921</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>19.06087318550538</v>
+        <v>14.14828693055786</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.54888370205292</v>
+        <v>0.2998348168701576</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0261110414740232</v>
+        <v>0.2779997355795514</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6757</v>
+        <v>6790</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>台灣虎航-創</t>
+          <t>永豐實</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>196.3617246949875</v>
+        <v>201.3433314012784</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>56</v>
+        <v>37.9</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>48.34880300169042</v>
+        <v>35.57018055996438</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>11.75512987473721</v>
+        <v>19.06087318550538</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.6524631320011687</v>
+        <v>0.54888370205292</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,48 +6294,48 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0253399523182022</v>
+        <v>-0.0261110414740232</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6667</v>
+        <v>6757</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>台灣虎航-創</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>185.0845043099733</v>
+        <v>196.3617246949875</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>222</v>
+        <v>56</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G111" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>38.25904583020812</v>
+        <v>48.34880300169042</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>26.86517908304493</v>
+        <v>11.75512987473721</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.8349762433741935</v>
+        <v>0.6524631320011687</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,48 +6347,48 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.6410082331557998</v>
+        <v>-0.0253399523182022</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6573</v>
+        <v>6667</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>虹揚-KY</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>180.9999152164346</v>
+        <v>185.0845043099733</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>16.45</v>
+        <v>222</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G112" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>40.9249767188394</v>
+        <v>38.25904583020812</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>14.85235303881452</v>
+        <v>26.86517908304493</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.4389146556884939</v>
+        <v>0.8349762433741935</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,48 +6400,48 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.08126752398973019</v>
+        <v>0.6410082331557998</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6561</v>
+        <v>6573</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>虹揚-KY</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>176.7262751331408</v>
+        <v>180.9999152164346</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>320</v>
+        <v>16.45</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G113" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>41.79081351616983</v>
+        <v>40.9249767188394</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>13.91104868318157</v>
+        <v>14.85235303881452</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>1.369563003397402</v>
+        <v>0.4389146556884939</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.4854780209325167</v>
+        <v>-0.08126752398973019</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6556</v>
+        <v>6561</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>勝品</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>174.1076277047995</v>
+        <v>176.7262751331408</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>59.1</v>
+        <v>320</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>32.85600619969021</v>
+        <v>41.79081351616983</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>23.100326704928</v>
+        <v>13.91104868318157</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.8447210296181815</v>
+        <v>1.369563003397402</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.4473183897035984</v>
+        <v>0.4854780209325167</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6725</v>
+        <v>6556</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>矽科宏晟</t>
+          <t>勝品</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>166.4623594299118</v>
+        <v>174.1076277047995</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>238</v>
+        <v>59.1</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>34.72140823297465</v>
+        <v>32.85600619969021</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>24.65817778554164</v>
+        <v>23.100326704928</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.8795495370593626</v>
+        <v>0.8447210296181815</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1605444997505287</v>
+        <v>-0.4473183897035984</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6569,38 +6569,38 @@
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6794</v>
+        <v>6725</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>矽科宏晟</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>165.1171184865939</v>
+        <v>166.4623594299118</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>68.8</v>
+        <v>238</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G116" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>24.64589243797722</v>
+        <v>34.72140823297465</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>16.85125059311614</v>
+        <v>24.65817778554164</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>1.686321062690677</v>
+        <v>0.8795495370593626</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.5454024850018246</v>
+        <v>-0.1605444997505287</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6625</v>
+        <v>6794</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>161.2482611190787</v>
+        <v>165.1171184865939</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>77.3</v>
+        <v>68.8</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>52.97446421272409</v>
+        <v>24.64589243797722</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>12.88979239576747</v>
+        <v>16.85125059311614</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4144315907900274</v>
+        <v>1.686321062690677</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.2127068229483267</v>
+        <v>-0.5454024850018246</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6541</v>
+        <v>6625</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>必應</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>155.7282608521141</v>
+        <v>161.2482611190787</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>37.3</v>
+        <v>77.3</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>41.74081981412946</v>
+        <v>52.97446421272409</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>8.837137102480504</v>
+        <v>12.88979239576747</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.5016035368622297</v>
+        <v>0.4144315907900274</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0235797533809138</v>
+        <v>0.2127068229483267</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6614</v>
+        <v>6541</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>127.2398745234386</v>
+        <v>155.7282608521141</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>36.05</v>
+        <v>37.3</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>34.66538554930089</v>
+        <v>41.74081981412946</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>14.17410226352386</v>
+        <v>8.837137102480504</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4429753065131716</v>
+        <v>0.5016035368622297</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.0441616404204838</v>
+        <v>0.0235797533809138</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6781,38 +6781,38 @@
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6732</v>
+        <v>6614</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>昇佳電子</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>124.0268418814192</v>
+        <v>127.2398745234386</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>158</v>
+        <v>36.05</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G120" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>43.05787210695334</v>
+        <v>34.66538554930089</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>19.9105804958498</v>
+        <v>14.17410226352386</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.6273625023937905</v>
+        <v>0.4429753065131716</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,48 +6824,48 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.170692809927619</v>
+        <v>0.0441616404204838</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6776</v>
+        <v>6732</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>昇佳電子</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>119.0000941388561</v>
+        <v>124.0268418814192</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>53.6</v>
+        <v>158</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G121" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>45.27027351278529</v>
+        <v>43.05787210695334</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>18.93232410566946</v>
+        <v>19.9105804958498</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.5997270703153056</v>
+        <v>0.6273625023937905</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.1458669201707986</v>
+        <v>-0.170692809927619</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6754</v>
+        <v>6776</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>116.2180106972832</v>
+        <v>119.0000941388561</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>41.55</v>
+        <v>53.6</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>40.0081267812346</v>
+        <v>45.27027351278529</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>8.833402784507792</v>
+        <v>18.93232410566946</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.5467694616906598</v>
+        <v>0.5997270703153056</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.0127949129206118</v>
+        <v>0.1458669201707986</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6641</v>
+        <v>6754</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>基士德-KY</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>112.3571782363066</v>
+        <v>116.2180106972832</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>18.1</v>
+        <v>41.55</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>54.29513512300322</v>
+        <v>40.0081267812346</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>9.363143928272716</v>
+        <v>8.833402784507792</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.2448373808626353</v>
+        <v>0.5467694616906598</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0586251273934338</v>
+        <v>0.0127949129206118</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6838</v>
+        <v>6641</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>基士德-KY</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>105.5294906835739</v>
+        <v>112.3571782363066</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>22.95</v>
+        <v>18.1</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>39.31739066789767</v>
+        <v>54.29513512300322</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>10.99112255579644</v>
+        <v>9.363143928272716</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.2571716159304169</v>
+        <v>0.2448373808626353</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.0343467113302833</v>
+        <v>0.0586251273934338</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,21 +7046,21 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6552</v>
+        <v>6838</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>85.64302450384848</v>
+        <v>105.5294906835739</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>24.7</v>
+        <v>22.95</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>42.67246788611487</v>
+        <v>39.31739066789767</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18.51320631289275</v>
+        <v>10.99112255579644</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.3740901079820794</v>
+        <v>0.2571716159304169</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.2800822590224472</v>
+        <v>-0.0343467113302833</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,52 +7099,105 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
+        <v>6552</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>易華電</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>85.64302450384848</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>42.67246788611487</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>18.51320631289275</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.3740901079820794</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>0.2800822590224472</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>6823</v>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>濾能</t>
         </is>
       </c>
-      <c r="C126" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D126" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>67.21719010208515</v>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>62.8</v>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>43.40787337338165</v>
       </c>
-      <c r="I126" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>12.9564988501562</v>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.3928287632169864</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N126" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>0.0579625711740523</v>
       </c>
-      <c r="O126" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>